<commit_message>
semantic v2: regenerate metric inventory (binding dimensions, Meta-only dimension notes)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/METRIC_INVENTORY.xlsx
+++ b/doc/METRIC_INVENTORY.xlsx
@@ -480,14 +480,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-04 07:23 UTC by scripts/build_metric_inventory_v2.py (Seleric_Agent_Core c811799).</t>
+          <t>Generated 2026-10-04 08:53 UTC by scripts/build_metric_inventory_v2.py (Seleric_Agent_Core a00155f).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>catalogue_v2 003767f63786: 109 metrics, 18 views, 122 dimensions, 5 hierarchies, 27 concepts, 414 glossary terms, 146 retired v1 ids; agent registry 89 entries.</t>
+          <t>catalogue_v2 f22a6b856d2b: 109 metrics, 18 views, 122 dimensions, 5 hierarchies, 27 concepts, 414 glossary terms, 146 retired v1 ids; agent registry 89 entries.</t>
         </is>
       </c>
     </row>
@@ -21627,7 +21627,7 @@
         <v>931</v>
       </c>
       <c r="AA25" t="n">
-        <v>1553</v>
+        <v>1552</v>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
@@ -21744,7 +21744,7 @@
         <v>339</v>
       </c>
       <c r="AA26" t="n">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="AB26" t="inlineStr">
         <is>
@@ -21865,7 +21865,7 @@
         <v>0.364125</v>
       </c>
       <c r="AA27" t="n">
-        <v>0.320026</v>
+        <v>0.319588</v>
       </c>
       <c r="AB27" t="inlineStr">
         <is>
@@ -29000,7 +29000,7 @@
         </is>
       </c>
       <c r="Z85" t="n">
-        <v>8.563442</v>
+        <v>8.563385</v>
       </c>
       <c r="AA85" t="n">
         <v>4.977296</v>
@@ -29246,7 +29246,7 @@
         </is>
       </c>
       <c r="Z87" t="n">
-        <v>48982</v>
+        <v>48981</v>
       </c>
       <c r="AA87" t="n">
         <v>51866</v>
@@ -29738,7 +29738,7 @@
         </is>
       </c>
       <c r="Z91" t="n">
-        <v>764457</v>
+        <v>764456</v>
       </c>
       <c r="AA91" t="n">
         <v>665923</v>
@@ -29859,7 +29859,7 @@
         </is>
       </c>
       <c r="Z92" t="n">
-        <v>0.342937</v>
+        <v>0.342925</v>
       </c>
       <c r="AA92" t="n">
         <v>0.257829</v>
@@ -31506,7 +31506,7 @@
         </is>
       </c>
       <c r="Z106" t="n">
-        <v>0.657063</v>
+        <v>0.657075</v>
       </c>
       <c r="AA106" t="n">
         <v>0.742171</v>
@@ -31736,7 +31736,7 @@
         </is>
       </c>
       <c r="Z108" t="n">
-        <v>47983</v>
+        <v>47984</v>
       </c>
       <c r="AA108" t="n">
         <v>51363</v>
@@ -31849,7 +31849,7 @@
         </is>
       </c>
       <c r="Z109" t="n">
-        <v>104175</v>
+        <v>104176</v>
       </c>
       <c r="AA109" t="n">
         <v>156501</v>
@@ -38677,7 +38677,7 @@
         </is>
       </c>
       <c r="E287" t="n">
-        <v>0.843764</v>
+        <v>0.843797</v>
       </c>
     </row>
     <row r="288">
@@ -38769,7 +38769,7 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>0.703501</v>
+        <v>0.703521</v>
       </c>
     </row>
     <row r="292">
@@ -40964,10 +40964,10 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>48982</v>
+        <v>48981</v>
       </c>
       <c r="F30" t="n">
-        <v>48982</v>
+        <v>48981</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -44162,10 +44162,10 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>0.657063</v>
+        <v>0.657075</v>
       </c>
       <c r="F133" t="n">
-        <v>0.657063</v>
+        <v>0.657075</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -45853,7 +45853,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Age bucket.</t>
+          <t>Meta audience breakdown (breakdown_type age_and_gender); Meta delivery only — Google reports no audience breakdowns. Age bucket.</t>
         </is>
       </c>
     </row>
@@ -45987,7 +45987,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Which breakdown the row belongs to (age_gender, placement, device, region …).</t>
+          <t>Meta audience breakdown (one breakdown_type per query); Meta delivery only — Google reports no audience breakdowns. Which breakdown the row belongs to (age_gender, placement, device, region …).</t>
         </is>
       </c>
     </row>
@@ -46311,7 +46311,7 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Country.</t>
+          <t>Meta audience breakdown (never populated — not answerable); Meta delivery only — Google reports no audience breakdowns. Country.</t>
         </is>
       </c>
     </row>
@@ -46467,7 +46467,7 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>mobile | desktop.</t>
+          <t>Meta audience breakdown (breakdown_type platform_device); Meta delivery only — Google reports no audience breakdowns. mobile | desktop.</t>
         </is>
       </c>
     </row>
@@ -46825,7 +46825,7 @@
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Gender.</t>
+          <t>Meta audience breakdown (breakdown_type age_and_gender); Meta delivery only — Google reports no audience breakdowns. Gender.</t>
         </is>
       </c>
     </row>
@@ -46993,7 +46993,7 @@
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Impression device.</t>
+          <t>Meta audience breakdown (breakdown_type placement); Meta delivery only — Google reports no audience breakdowns. Impression device.</t>
         </is>
       </c>
     </row>
@@ -47909,7 +47909,7 @@
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Placement (feed, story, reels …).</t>
+          <t>Meta audience breakdown (breakdown_type placement); Meta delivery only — Google reports no audience breakdowns. Placement (feed, story, reels …).</t>
         </is>
       </c>
     </row>
@@ -48077,7 +48077,7 @@
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>facebook | instagram | audience_network | messenger.</t>
+          <t>Meta audience breakdown (breakdown_type publisher_platform, placement, platform_device); Meta delivery only — Google reports no audience breakdowns. facebook | instagram | audience_network | messenger.</t>
         </is>
       </c>
     </row>
@@ -48159,7 +48159,7 @@
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Region / state.</t>
+          <t>Meta audience breakdown (breakdown_type region); Meta delivery only — Google reports no audience breakdowns. Region / state.</t>
         </is>
       </c>
     </row>

</xml_diff>